<commit_message>
Sync website content 2026-05-25 13:24
</commit_message>
<xml_diff>
--- a/组合介绍/report_assets/factors/workbooks/1-Microsoft_Excel_Worksheet1.xlsx
+++ b/组合介绍/report_assets/factors/workbooks/1-Microsoft_Excel_Worksheet1.xlsx
@@ -7,7 +7,7 @@
     <workbookView windowHeight="15800" windowWidth="28040" xWindow="4240" yWindow="640"/>
   </bookViews>
   <sheets>
-    <sheet name="10vrt3" sheetId="2" r:id="rId5"/>
+    <sheet name="YGAvm2" sheetId="2" r:id="rId5"/>
   </sheets>
   <calcPr calcMode="auto"/>
   <extLst>
@@ -94,14 +94,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -127,17 +120,14 @@
   <cellStyleXfs count="1">
     <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="false" applyNumberFormat="false" applyProtection="false" borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf applyAlignment="false" applyBorder="false" applyFill="false" applyFont="false" applyNumberFormat="false" applyProtection="false" borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
+      <alignment horizontal="left" vertical="center" wrapText="true"/>
     </xf>
     <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="2" fillId="0" fontId="2" numFmtId="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="true"/>
-    </xf>
-    <xf applyAlignment="true" applyBorder="false" applyFill="false" applyFont="true" applyNumberFormat="false" applyProtection="false" borderId="3" fillId="0" fontId="2" numFmtId="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="true"/>
     </xf>
   </cellXfs>
@@ -459,71 +449,74 @@
   </sheetPr>
   <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="14" defaultRowHeight="19"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" max="1" min="1" style="0" width="25"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="str">
-        <v>排名</v>
+        <v>指标名称</v>
       </c>
       <c r="B1" s="1" t="str">
-        <v>入选指标</v>
+        <v>最大相关性</v>
       </c>
       <c r="C1" s="1" t="str">
-        <v>经济含义</v>
+        <v>领先月数</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2">
+      <c r="A2" s="2" t="str">
+        <v>汽车：产量：当月值</v>
+      </c>
+      <c r="B2" s="2">
+        <v>0.654</v>
+      </c>
+      <c r="C2" s="2">
         <v>1</v>
-      </c>
-      <c r="B2" s="3" t="str">
-        <v>汽车产量：当月值</v>
-      </c>
-      <c r="C2" s="3" t="str">
-        <v>反映制造业和耐用品消费景气</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2">
-        <v>2</v>
-      </c>
-      <c r="B3" s="3" t="str">
-        <v>挖掘机产量：当月值</v>
-      </c>
-      <c r="C3" s="3" t="str">
-        <v>反映工程机械和基建施工需求</v>
+      <c r="A3" s="2" t="str">
+        <v>挖掘机：产量：当月值</v>
+      </c>
+      <c r="B3" s="2">
+        <v>0.632</v>
+      </c>
+      <c r="C3" s="2">
+        <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2">
-        <v>3</v>
-      </c>
-      <c r="B4" s="3" t="str">
-        <v>基础设施建设投资：折算当月值</v>
-      </c>
-      <c r="C4" s="3" t="str">
-        <v>反映基建投资强度</v>
+      <c r="A4" s="2" t="str">
+        <v>固定资产投资 (不含农户) 完成额：基础设施建设投资：折算当月值</v>
+      </c>
+      <c r="B4" s="2">
+        <v>0.503</v>
+      </c>
+      <c r="C4" s="2">
+        <v>4</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2">
-        <v>4</v>
-      </c>
-      <c r="B5" s="3" t="str">
+      <c r="A5" s="2" t="str">
         <v>发电量：当月值</v>
       </c>
-      <c r="C5" s="3" t="str">
-        <v>反映工业生产和用电需求</v>
+      <c r="B5" s="2">
+        <v>0.44</v>
+      </c>
+      <c r="C5" s="2">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2">
-        <v>5</v>
-      </c>
-      <c r="B6" s="3" t="str">
-        <v>房地产建筑工程投资：折算当月值</v>
-      </c>
-      <c r="C6" s="3" t="str">
-        <v>反映地产施工链条景气</v>
+      <c r="A6" s="2" t="str">
+        <v>房地产开发投资完成额：建筑工程：折算当月值</v>
+      </c>
+      <c r="B6" s="2">
+        <v>0.291</v>
+      </c>
+      <c r="C6" s="2">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>